<commit_message>
fix(smd): preserve legacy workbook structures in import adapters
</commit_message>
<xml_diff>
--- a/smd-process-control/tests/fixtures/ict-sample.xlsx
+++ b/smd-process-control/tests/fixtures/ict-sample.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data HS Công Đoạn ICT" sheetId="1" r:id="R693211c8bba04d4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data HS Công Đoạn ICT" sheetId="1" r:id="R3d893bca1e3d4c0a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -271,107 +271,324 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="14" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="14" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="14" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="14" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="14" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="14" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="14" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="14" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="14" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="14" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="14" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="14" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="14" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="14" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="14" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="14" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="4">
-      <x:c r="A4" s="3" t="str">
-        <x:v>ICT daily performance</x:v>
-      </x:c>
+      <x:c r="B4" s="3" t="str">
+        <x:v>Data Theo Dõi Hiệu Suất công đoạn ICT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="B5" s="7"/>
+      <x:c r="C5" s="7" t="str">
+        <x:v>Ngày</x:v>
+      </x:c>
+      <x:c r="D5" s="7" t="str">
+        <x:v>Ca</x:v>
+      </x:c>
+      <x:c r="E5" s="7" t="str">
+        <x:v>Model</x:v>
+      </x:c>
+      <x:c r="F5" s="7"/>
+      <x:c r="G5" s="7" t="str">
+        <x:v>Time</x:v>
+      </x:c>
+      <x:c r="H5" s="7" t="str">
+        <x:v>Input</x:v>
+      </x:c>
+      <x:c r="I5" s="7" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="J5" s="7"/>
+      <x:c r="K5" s="7"/>
+      <x:c r="L5" s="7"/>
+      <x:c r="M5" s="7" t="str">
+        <x:v>NG</x:v>
+      </x:c>
+      <x:c r="N5" s="7"/>
+      <x:c r="O5" s="7"/>
+      <x:c r="P5" s="7"/>
+      <x:c r="Q5" s="7" t="str">
+        <x:v>Chi Tiết Lỗi</x:v>
+      </x:c>
+      <x:c r="R5" s="7"/>
+      <x:c r="S5" s="7"/>
+      <x:c r="T5" s="7"/>
+      <x:c r="U5" s="7"/>
+      <x:c r="V5" s="7"/>
+      <x:c r="W5" s="7"/>
+      <x:c r="X5" s="7"/>
+      <x:c r="Y5" s="7"/>
+      <x:c r="Z5" s="7"/>
+      <x:c r="AA5" s="7"/>
+      <x:c r="AB5" s="7"/>
+      <x:c r="AC5" s="7"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="B6" s="7"/>
+      <x:c r="C6" s="7"/>
+      <x:c r="D6" s="7"/>
+      <x:c r="E6" s="7"/>
+      <x:c r="F6" s="7"/>
+      <x:c r="G6" s="7"/>
+      <x:c r="H6" s="7"/>
+      <x:c r="I6" s="7"/>
+      <x:c r="J6" s="7"/>
+      <x:c r="K6" s="7"/>
+      <x:c r="L6" s="7"/>
+      <x:c r="M6" s="7"/>
+      <x:c r="N6" s="7"/>
+      <x:c r="O6" s="7"/>
+      <x:c r="P6" s="7"/>
+      <x:c r="Q6" s="7" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="R6" s="7"/>
+      <x:c r="S6" s="7"/>
+      <x:c r="T6" s="7"/>
+      <x:c r="U6" s="7"/>
+      <x:c r="V6" s="7"/>
+      <x:c r="W6" s="7"/>
+      <x:c r="X6" s="7"/>
+      <x:c r="Y6" s="7"/>
+      <x:c r="Z6" s="7"/>
+      <x:c r="AA6" s="7"/>
+      <x:c r="AB6" s="7"/>
+      <x:c r="AC6" s="7"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="7" t="str">
-        <x:v>Date</x:v>
-      </x:c>
-      <x:c r="B7" s="7" t="str">
-        <x:v>Shift</x:v>
-      </x:c>
-      <x:c r="C7" s="7" t="str">
-        <x:v>Time</x:v>
-      </x:c>
-      <x:c r="D7" s="7" t="str">
-        <x:v>Line</x:v>
-      </x:c>
-      <x:c r="E7" s="7" t="str">
-        <x:v>Model</x:v>
-      </x:c>
-      <x:c r="F7" s="7" t="str">
-        <x:v>Input</x:v>
-      </x:c>
-      <x:c r="G7" s="7" t="str">
-        <x:v>OK</x:v>
-      </x:c>
-      <x:c r="H7" s="7" t="str">
-        <x:v>NG</x:v>
-      </x:c>
+      <x:c r="B7" s="7"/>
+      <x:c r="C7" s="7"/>
+      <x:c r="D7" s="7"/>
+      <x:c r="E7" s="7"/>
+      <x:c r="F7" s="7"/>
+      <x:c r="G7" s="7"/>
+      <x:c r="H7" s="7"/>
       <x:c r="I7" s="7" t="str">
-        <x:v>Yield</x:v>
-      </x:c>
+        <x:v>Trước CF</x:v>
+      </x:c>
+      <x:c r="J7" s="7"/>
+      <x:c r="K7" s="7" t="str">
+        <x:v>Sau CF</x:v>
+      </x:c>
+      <x:c r="L7" s="7"/>
+      <x:c r="M7" s="7" t="str">
+        <x:v>Trước CF</x:v>
+      </x:c>
+      <x:c r="N7" s="7"/>
+      <x:c r="O7" s="7" t="str">
+        <x:v>Sau CF</x:v>
+      </x:c>
+      <x:c r="P7" s="7"/>
+      <x:c r="Q7" s="7"/>
+      <x:c r="R7" s="7"/>
+      <x:c r="S7" s="7"/>
+      <x:c r="T7" s="7"/>
+      <x:c r="U7" s="7"/>
+      <x:c r="V7" s="7"/>
+      <x:c r="W7" s="7"/>
+      <x:c r="X7" s="7"/>
+      <x:c r="Y7" s="7"/>
+      <x:c r="Z7" s="7"/>
+      <x:c r="AA7" s="7"/>
+      <x:c r="AB7" s="7"/>
+      <x:c r="AC7" s="7"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>27.07.2026</x:v>
-      </x:c>
-      <x:c r="B8" t="str">
-        <x:v>DAY</x:v>
-      </x:c>
-      <x:c r="C8"/>
-      <x:c r="D8" t="str">
-        <x:v>Line 1</x:v>
-      </x:c>
+      <x:c r="B8"/>
+      <x:c r="C8" t="str">
+        <x:v>TOTAL(Tháng)</x:v>
+      </x:c>
+      <x:c r="D8"/>
       <x:c r="E8" t="str">
         <x:v>MODEL-A</x:v>
       </x:c>
-      <x:c r="F8" t="n">
+      <x:c r="F8"/>
+      <x:c r="G8"/>
+      <x:c r="H8" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="G8" t="n">
+      <x:c r="I8" t="n">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="H8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I8" t="n">
-        <x:f>G8/F8</x:f>
+      <x:c r="J8" t="n">
         <x:v>0.95</x:v>
       </x:c>
+      <x:c r="K8" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="L8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N8" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="O8" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" t="str">
+      <x:c r="B9"/>
+      <x:c r="C9" t="str">
         <x:v>27.07.2026</x:v>
       </x:c>
-      <x:c r="B9" t="str">
+      <x:c r="D9" t="str">
         <x:v>DAY</x:v>
       </x:c>
-      <x:c r="C9"/>
-      <x:c r="D9" t="str">
-        <x:v>TOTAL</x:v>
-      </x:c>
       <x:c r="E9"/>
-      <x:c r="F9" t="n">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="G9" t="n">
-        <x:v>33</x:v>
+      <x:c r="F9" t="str">
+        <x:v>MODEL-A</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>A</x:v>
       </x:c>
       <x:c r="H9" t="n">
-        <x:v>2</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="I9" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>#DIV/0!</x:v>
+      </x:c>
+      <x:c r="K9" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="L9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N9" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="O9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="B10"/>
+      <x:c r="C10"/>
+      <x:c r="D10"/>
+      <x:c r="E10"/>
+      <x:c r="F10"/>
+      <x:c r="G10" t="str">
+        <x:v>TTL</x:v>
+      </x:c>
+      <x:c r="H10" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="I10" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J10" t="n">
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="K10" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="L10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N10" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="O10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="B11"/>
+      <x:c r="C11" t="str">
+        <x:v>27.07.2026</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>DAY</x:v>
+      </x:c>
+      <x:c r="E11"/>
+      <x:c r="F11"/>
+      <x:c r="G11" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J11" t="n">
         <x:v>0.9</x:v>
       </x:c>
+      <x:c r="K11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="L11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N11" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="O11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="B12"/>
+      <x:c r="C12"/>
+      <x:c r="D12"/>
+      <x:c r="E12"/>
+      <x:c r="F12"/>
+      <x:c r="G12"/>
+      <x:c r="H12"/>
+      <x:c r="I12"/>
+      <x:c r="J12"/>
+      <x:c r="K12"/>
+      <x:c r="L12"/>
+      <x:c r="M12"/>
+      <x:c r="N12"/>
+      <x:c r="O12"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A4:I4"/>
+    <x:mergeCell ref="B4:AC4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>